<commit_message>
Adding latest flooding data and updated to local-env-data
</commit_message>
<xml_diff>
--- a/datasets/local-data/FoE-local-env-data-MAYORAL-2026.xlsx
+++ b/datasets/local-data/FoE-local-env-data-MAYORAL-2026.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="99">
   <si>
     <t xml:space="preserve">Metromayor code</t>
   </si>
@@ -66,6 +66,9 @@
   </si>
   <si>
     <t xml:space="preserve">EV chargers: 2030 target</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Electric plugin vehicles</t>
   </si>
   <si>
     <t xml:space="preserve">Commuters: bicycle (%)</t>
@@ -749,6 +752,7 @@
     <col min="52" max="52" width="20.71" hidden="0" customWidth="1"/>
     <col min="53" max="53" width="20.71" hidden="0" customWidth="1"/>
     <col min="54" max="54" width="20.71" hidden="0" customWidth="1"/>
+    <col min="55" max="55" width="20.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -914,16 +918,19 @@
       <c r="BB1" s="1" t="s">
         <v>53</v>
       </c>
+      <c r="BC1" s="1" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D2" s="4" t="n">
         <v>0.278</v>
@@ -970,124 +977,127 @@
       <c r="R2" s="5" t="n">
         <v>12960</v>
       </c>
-      <c r="S2" s="4" t="n">
+      <c r="S2" s="5" t="n">
+        <v>39847</v>
+      </c>
+      <c r="T2" s="4" t="n">
         <v>0.022</v>
       </c>
-      <c r="T2" s="4" t="n">
+      <c r="U2" s="4" t="n">
         <v>0.288</v>
       </c>
-      <c r="U2" s="5" t="n">
+      <c r="V2" s="5" t="n">
         <v>335200</v>
       </c>
-      <c r="V2" s="5" t="n">
+      <c r="W2" s="5" t="n">
         <v>271915</v>
       </c>
-      <c r="W2" s="5" t="n">
+      <c r="X2" s="5" t="n">
         <v>0.66</v>
       </c>
-      <c r="X2" s="5" t="n">
+      <c r="Y2" s="5" t="n">
         <v>46120</v>
       </c>
-      <c r="Y2" s="5" t="n">
+      <c r="Z2" s="5" t="n">
         <v>9507</v>
       </c>
-      <c r="Z2" s="5" t="n">
+      <c r="AA2" s="5" t="n">
         <v>59.9</v>
       </c>
-      <c r="AA2" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="AB2" s="5" t="n">
+      <c r="AB2" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC2" s="5" t="n">
         <v>78010</v>
       </c>
-      <c r="AC2" s="5" t="n">
+      <c r="AD2" s="5" t="n">
         <v>53290</v>
       </c>
-      <c r="AD2" s="5" t="n">
+      <c r="AE2" s="5" t="n">
         <v>33840</v>
       </c>
-      <c r="AE2" s="5" t="n">
+      <c r="AF2" s="5" t="n">
         <v>163610</v>
       </c>
-      <c r="AF2" s="5" t="n">
+      <c r="AG2" s="5" t="n">
         <v>116470</v>
       </c>
-      <c r="AG2" s="5" t="n">
+      <c r="AH2" s="5" t="n">
         <v>71060</v>
       </c>
-      <c r="AH2" s="5" t="n">
+      <c r="AI2" s="5" t="n">
         <v>115</v>
       </c>
-      <c r="AI2" s="4" t="n">
+      <c r="AJ2" s="4" t="n">
         <v>0.326</v>
       </c>
-      <c r="AJ2" s="5" t="n">
+      <c r="AK2" s="5" t="n">
         <v>1016984</v>
       </c>
-      <c r="AK2" s="5" t="n">
+      <c r="AL2" s="5" t="n">
         <v>29.3</v>
       </c>
-      <c r="AL2" s="5" t="n">
+      <c r="AM2" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="AM2" s="5" t="n">
+      <c r="AN2" s="5" t="n">
         <v>278</v>
       </c>
-      <c r="AN2" s="5" t="n">
+      <c r="AO2" s="5" t="n">
         <v>45</v>
       </c>
-      <c r="AO2" s="4" t="n">
+      <c r="AP2" s="4" t="n">
         <v>0.151</v>
       </c>
-      <c r="AP2" s="4" t="n">
+      <c r="AQ2" s="4" t="n">
         <v>0.413</v>
       </c>
-      <c r="AQ2" s="4" t="n">
+      <c r="AR2" s="4" t="n">
         <v>0.785</v>
       </c>
-      <c r="AR2" s="5" t="n">
+      <c r="AS2" s="5" t="n">
         <v>818</v>
       </c>
-      <c r="AS2" s="5" t="n">
+      <c r="AT2" s="5" t="n">
         <v>22288</v>
       </c>
-      <c r="AT2" s="5" t="n">
+      <c r="AU2" s="5" t="n">
         <v>93292.11</v>
       </c>
-      <c r="AU2" s="4" t="n">
+      <c r="AV2" s="4" t="n">
         <v>0.504</v>
       </c>
-      <c r="AV2" s="4" t="n">
+      <c r="AW2" s="4" t="n">
         <v>0.538</v>
       </c>
-      <c r="AW2" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="AX2" s="4" t="n">
+      <c r="AX2" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="AY2" s="4" t="n">
         <v>0.7793</v>
       </c>
-      <c r="AY2" s="4" t="n">
+      <c r="AZ2" s="4" t="n">
         <v>0.656</v>
       </c>
-      <c r="AZ2" s="4" t="n">
+      <c r="BA2" s="4" t="n">
         <v>0.7918</v>
       </c>
-      <c r="BA2" s="5" t="n">
+      <c r="BB2" s="5" t="n">
         <v>657</v>
       </c>
-      <c r="BB2" s="4" t="n">
+      <c r="BC2" s="4" t="n">
         <v>-0.326173759624042</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D3" s="4" t="n">
         <v>0.241</v>
@@ -1134,124 +1144,127 @@
       <c r="R3" s="5" t="n">
         <v>6184</v>
       </c>
-      <c r="S3" s="4" t="n">
+      <c r="S3" s="5" t="n">
+        <v>10689</v>
+      </c>
+      <c r="T3" s="4" t="n">
         <v>0.017</v>
       </c>
-      <c r="T3" s="4" t="n">
+      <c r="U3" s="4" t="n">
         <v>0.226</v>
       </c>
-      <c r="U3" s="5" t="n">
+      <c r="V3" s="5" t="n">
         <v>3634900</v>
       </c>
-      <c r="V3" s="5" t="n">
+      <c r="W3" s="5" t="n">
         <v>827771</v>
       </c>
-      <c r="W3" s="5" t="n">
+      <c r="X3" s="5" t="n">
         <v>0.39</v>
       </c>
-      <c r="X3" s="5" t="n">
+      <c r="Y3" s="5" t="n">
         <v>35190</v>
       </c>
-      <c r="Y3" s="5" t="n">
+      <c r="Z3" s="5" t="n">
         <v>5785</v>
       </c>
-      <c r="Z3" s="5" t="n">
+      <c r="AA3" s="5" t="n">
         <v>354.2</v>
       </c>
-      <c r="AA3" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="AB3" s="5" t="n">
+      <c r="AB3" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="AC3" s="5" t="n">
         <v>34460</v>
       </c>
-      <c r="AC3" s="5" t="n">
+      <c r="AD3" s="5" t="n">
         <v>25860</v>
       </c>
-      <c r="AD3" s="5" t="n">
+      <c r="AE3" s="5" t="n">
         <v>14840</v>
       </c>
-      <c r="AE3" s="5" t="n">
+      <c r="AF3" s="5" t="n">
         <v>74090</v>
       </c>
-      <c r="AF3" s="5" t="n">
+      <c r="AG3" s="5" t="n">
         <v>54670</v>
       </c>
-      <c r="AG3" s="5" t="n">
+      <c r="AH3" s="5" t="n">
         <v>32750</v>
       </c>
-      <c r="AH3" s="5" t="n">
+      <c r="AI3" s="5" t="n">
         <v>65</v>
       </c>
-      <c r="AI3" s="4" t="n">
+      <c r="AJ3" s="4" t="n">
         <v>0.38</v>
       </c>
-      <c r="AJ3" s="5" t="n">
+      <c r="AK3" s="5" t="n">
         <v>527751</v>
       </c>
-      <c r="AK3" s="5" t="n">
+      <c r="AL3" s="5" t="n">
         <v>30.7</v>
       </c>
-      <c r="AL3" s="5" t="n">
+      <c r="AM3" s="5" t="n">
         <v>40.3</v>
       </c>
-      <c r="AM3" s="5" t="n">
+      <c r="AN3" s="5" t="n">
         <v>341</v>
       </c>
-      <c r="AN3" s="5" t="n">
+      <c r="AO3" s="5" t="n">
         <v>39</v>
       </c>
-      <c r="AO3" s="4" t="n">
+      <c r="AP3" s="4" t="n">
         <v>0.158</v>
       </c>
-      <c r="AP3" s="4" t="n">
+      <c r="AQ3" s="4" t="n">
         <v>0.39</v>
       </c>
-      <c r="AQ3" s="4" t="n">
+      <c r="AR3" s="4" t="n">
         <v>0.765</v>
       </c>
-      <c r="AR3" s="5" t="n">
+      <c r="AS3" s="5" t="n">
         <v>183</v>
       </c>
-      <c r="AS3" s="5" t="n">
+      <c r="AT3" s="5" t="n">
         <v>4724</v>
       </c>
-      <c r="AT3" s="5" t="n">
+      <c r="AU3" s="5" t="n">
         <v>28869.03</v>
       </c>
-      <c r="AU3" s="4" t="n">
+      <c r="AV3" s="4" t="n">
         <v>0.399</v>
       </c>
-      <c r="AV3" s="4" t="n">
+      <c r="AW3" s="4" t="n">
         <v>0.538</v>
       </c>
-      <c r="AW3" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="AX3" s="4" t="n">
+      <c r="AX3" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="AY3" s="4" t="n">
         <v>0.7476</v>
       </c>
-      <c r="AY3" s="4" t="n">
+      <c r="AZ3" s="4" t="n">
         <v>0.6296</v>
       </c>
-      <c r="AZ3" s="4" t="n">
+      <c r="BA3" s="4" t="n">
         <v>0.7631</v>
       </c>
-      <c r="BA3" s="5" t="n">
+      <c r="BB3" s="5" t="n">
         <v>174</v>
       </c>
-      <c r="BB3" s="4" t="n">
+      <c r="BC3" s="4" t="n">
         <v>-0.524922623692494</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D4" s="4" t="n">
         <v>0.275</v>
@@ -1298,124 +1311,127 @@
       <c r="R4" s="5" t="n">
         <v>10557</v>
       </c>
-      <c r="S4" s="4" t="n">
+      <c r="S4" s="5" t="n">
+        <v>36583</v>
+      </c>
+      <c r="T4" s="4" t="n">
         <v>0.013</v>
       </c>
-      <c r="T4" s="4" t="n">
+      <c r="U4" s="4" t="n">
         <v>0.222</v>
       </c>
-      <c r="U4" s="5" t="n">
+      <c r="V4" s="5" t="n">
         <v>1086800</v>
       </c>
-      <c r="V4" s="5" t="n">
+      <c r="W4" s="5" t="n">
         <v>495930</v>
       </c>
-      <c r="W4" s="5" t="n">
+      <c r="X4" s="5" t="n">
         <v>0.56</v>
       </c>
-      <c r="X4" s="5" t="n">
+      <c r="Y4" s="5" t="n">
         <v>42290</v>
       </c>
-      <c r="Y4" s="5" t="n">
+      <c r="Z4" s="5" t="n">
         <v>8035</v>
       </c>
-      <c r="Z4" s="5" t="n">
+      <c r="AA4" s="5" t="n">
         <v>127.8</v>
       </c>
-      <c r="AA4" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="AB4" s="5" t="n">
+      <c r="AB4" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="AC4" s="5" t="n">
         <v>53140</v>
       </c>
-      <c r="AC4" s="5" t="n">
+      <c r="AD4" s="5" t="n">
         <v>47490</v>
       </c>
-      <c r="AD4" s="5" t="n">
+      <c r="AE4" s="5" t="n">
         <v>23590</v>
       </c>
-      <c r="AE4" s="5" t="n">
+      <c r="AF4" s="5" t="n">
         <v>102090</v>
       </c>
-      <c r="AF4" s="5" t="n">
+      <c r="AG4" s="5" t="n">
         <v>88950</v>
       </c>
-      <c r="AG4" s="5" t="n">
+      <c r="AH4" s="5" t="n">
         <v>45450</v>
       </c>
-      <c r="AH4" s="5" t="n">
+      <c r="AI4" s="5" t="n">
         <v>132</v>
       </c>
-      <c r="AI4" s="4" t="n">
+      <c r="AJ4" s="4" t="n">
         <v>0.439</v>
       </c>
-      <c r="AJ4" s="5" t="n">
+      <c r="AK4" s="5" t="n">
         <v>1070861</v>
       </c>
-      <c r="AK4" s="5" t="n">
+      <c r="AL4" s="5" t="n">
         <v>29.4</v>
       </c>
-      <c r="AL4" s="5" t="n">
+      <c r="AM4" s="5" t="n">
         <v>39.5</v>
       </c>
-      <c r="AM4" s="5" t="n">
+      <c r="AN4" s="5" t="n">
         <v>473</v>
       </c>
-      <c r="AN4" s="5" t="n">
+      <c r="AO4" s="5" t="n">
         <v>40</v>
       </c>
-      <c r="AO4" s="4" t="n">
+      <c r="AP4" s="4" t="n">
         <v>0.124</v>
       </c>
-      <c r="AP4" s="4" t="n">
+      <c r="AQ4" s="4" t="n">
         <v>0.544</v>
       </c>
-      <c r="AQ4" s="4" t="n">
+      <c r="AR4" s="4" t="n">
         <v>0.858</v>
       </c>
-      <c r="AR4" s="5" t="n">
+      <c r="AS4" s="5" t="n">
         <v>881</v>
       </c>
-      <c r="AS4" s="5" t="n">
+      <c r="AT4" s="5" t="n">
         <v>24909</v>
       </c>
-      <c r="AT4" s="5" t="n">
+      <c r="AU4" s="5" t="n">
         <v>115430.15</v>
       </c>
-      <c r="AU4" s="4" t="n">
+      <c r="AV4" s="4" t="n">
         <v>0.374</v>
       </c>
-      <c r="AV4" s="4" t="n">
+      <c r="AW4" s="4" t="n">
         <v>0.538</v>
       </c>
-      <c r="AW4" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="AX4" s="4" t="n">
+      <c r="AX4" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="AY4" s="4" t="n">
         <v>0.774</v>
       </c>
-      <c r="AY4" s="4" t="n">
+      <c r="AZ4" s="4" t="n">
         <v>0.6486</v>
       </c>
-      <c r="AZ4" s="4" t="n">
+      <c r="BA4" s="4" t="n">
         <v>0.7816</v>
       </c>
-      <c r="BA4" s="5" t="n">
+      <c r="BB4" s="5" t="n">
         <v>282</v>
       </c>
-      <c r="BB4" s="4" t="n">
+      <c r="BC4" s="4" t="n">
         <v>-0.281752783499</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D5" s="4" t="n">
         <v>0.266</v>
@@ -1462,124 +1478,127 @@
       <c r="R5" s="5" t="n">
         <v>6971</v>
       </c>
-      <c r="S5" s="4" t="n">
+      <c r="S5" s="5" t="n">
+        <v>21248</v>
+      </c>
+      <c r="T5" s="4" t="n">
         <v>0.021</v>
       </c>
-      <c r="T5" s="4" t="n">
+      <c r="U5" s="4" t="n">
         <v>0.295</v>
       </c>
-      <c r="U5" s="5" t="n">
+      <c r="V5" s="5" t="n">
         <v>101800</v>
       </c>
-      <c r="V5" s="5" t="n">
+      <c r="W5" s="5" t="n">
         <v>128085</v>
       </c>
-      <c r="W5" s="5" t="n">
+      <c r="X5" s="5" t="n">
         <v>0.56</v>
       </c>
-      <c r="X5" s="5" t="n">
+      <c r="Y5" s="5" t="n">
         <v>26980</v>
       </c>
-      <c r="Y5" s="5" t="n">
+      <c r="Z5" s="5" t="n">
         <v>3493</v>
       </c>
-      <c r="Z5" s="5" t="n">
+      <c r="AA5" s="5" t="n">
         <v>35.7</v>
       </c>
-      <c r="AA5" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="AB5" s="5" t="n">
+      <c r="AB5" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC5" s="5" t="n">
         <v>87860</v>
       </c>
-      <c r="AC5" s="5" t="n">
+      <c r="AD5" s="5" t="n">
         <v>58020</v>
       </c>
-      <c r="AD5" s="5" t="n">
+      <c r="AE5" s="5" t="n">
         <v>39590</v>
       </c>
-      <c r="AE5" s="5" t="n">
+      <c r="AF5" s="5" t="n">
         <v>138050</v>
       </c>
-      <c r="AF5" s="5" t="n">
+      <c r="AG5" s="5" t="n">
         <v>92650</v>
       </c>
-      <c r="AG5" s="5" t="n">
+      <c r="AH5" s="5" t="n">
         <v>62930</v>
       </c>
-      <c r="AH5" s="5" t="n">
+      <c r="AI5" s="5" t="n">
         <v>94</v>
       </c>
-      <c r="AI5" s="4" t="n">
+      <c r="AJ5" s="4" t="n">
         <v>0.468</v>
       </c>
-      <c r="AJ5" s="5" t="n">
+      <c r="AK5" s="5" t="n">
         <v>747561</v>
       </c>
-      <c r="AK5" s="5" t="n">
+      <c r="AL5" s="5" t="n">
         <v>29.4</v>
       </c>
-      <c r="AL5" s="5" t="n">
+      <c r="AM5" s="5" t="n">
         <v>37.6</v>
       </c>
-      <c r="AM5" s="5" t="n">
+      <c r="AN5" s="5" t="n">
         <v>352</v>
       </c>
-      <c r="AN5" s="5" t="n">
+      <c r="AO5" s="5" t="n">
         <v>37</v>
       </c>
-      <c r="AO5" s="4" t="n">
+      <c r="AP5" s="4" t="n">
         <v>0.137</v>
       </c>
-      <c r="AP5" s="4" t="n">
+      <c r="AQ5" s="4" t="n">
         <v>0.584</v>
       </c>
-      <c r="AQ5" s="4" t="n">
+      <c r="AR5" s="4" t="n">
         <v>0.87</v>
       </c>
-      <c r="AR5" s="5" t="n">
+      <c r="AS5" s="5" t="n">
         <v>158</v>
       </c>
-      <c r="AS5" s="5" t="n">
+      <c r="AT5" s="5" t="n">
         <v>4359</v>
       </c>
-      <c r="AT5" s="5" t="n">
+      <c r="AU5" s="5" t="n">
         <v>17994.52</v>
       </c>
-      <c r="AU5" s="4" t="n">
+      <c r="AV5" s="4" t="n">
         <v>0.347</v>
       </c>
-      <c r="AV5" s="4" t="n">
+      <c r="AW5" s="4" t="n">
         <v>0.538</v>
       </c>
-      <c r="AW5" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="AX5" s="4" t="n">
+      <c r="AX5" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="AY5" s="4" t="n">
         <v>0.7935</v>
       </c>
-      <c r="AY5" s="4" t="n">
+      <c r="AZ5" s="4" t="n">
         <v>0.6693</v>
       </c>
-      <c r="AZ5" s="4" t="n">
+      <c r="BA5" s="4" t="n">
         <v>0.8018</v>
       </c>
-      <c r="BA5" s="5" t="n">
+      <c r="BB5" s="5" t="n">
         <v>237</v>
       </c>
-      <c r="BB5" s="4" t="n">
+      <c r="BC5" s="4" t="n">
         <v>-0.38040422679372</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D6" s="4" t="n">
         <v>0.172</v>
@@ -1626,124 +1645,127 @@
       <c r="R6" s="5" t="n">
         <v>3072</v>
       </c>
-      <c r="S6" s="4" t="n">
+      <c r="S6" s="5" t="n">
+        <v>8717</v>
+      </c>
+      <c r="T6" s="4" t="n">
         <v>0.022</v>
       </c>
-      <c r="T6" s="4" t="n">
+      <c r="U6" s="4" t="n">
         <v>0.298</v>
       </c>
-      <c r="U6" s="5" t="n">
+      <c r="V6" s="5" t="n">
         <v>10365400</v>
       </c>
-      <c r="V6" s="5" t="n">
+      <c r="W6" s="5" t="n">
         <v>276423</v>
       </c>
-      <c r="W6" s="5" t="n">
+      <c r="X6" s="5" t="n">
         <v>0.21</v>
       </c>
-      <c r="X6" s="5" t="n">
+      <c r="Y6" s="5" t="n">
         <v>16600</v>
       </c>
-      <c r="Y6" s="5" t="n">
+      <c r="Z6" s="5" t="n">
         <v>2893</v>
       </c>
-      <c r="Z6" s="5" t="n">
+      <c r="AA6" s="5" t="n">
         <v>128</v>
       </c>
-      <c r="AA6" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="AB6" s="5" t="n">
+      <c r="AB6" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="AC6" s="5" t="n">
         <v>26930</v>
       </c>
-      <c r="AC6" s="5" t="n">
+      <c r="AD6" s="5" t="n">
         <v>18390</v>
       </c>
-      <c r="AD6" s="5" t="n">
+      <c r="AE6" s="5" t="n">
         <v>12270</v>
       </c>
-      <c r="AE6" s="5" t="n">
+      <c r="AF6" s="5" t="n">
         <v>51720</v>
       </c>
-      <c r="AF6" s="5" t="n">
+      <c r="AG6" s="5" t="n">
         <v>35240</v>
       </c>
-      <c r="AG6" s="5" t="n">
+      <c r="AH6" s="5" t="n">
         <v>23670</v>
       </c>
-      <c r="AH6" s="5" t="n">
+      <c r="AI6" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="AI6" s="4" t="n">
+      <c r="AJ6" s="4" t="n">
         <v>0.101</v>
       </c>
-      <c r="AJ6" s="5" t="n">
+      <c r="AK6" s="5" t="n">
         <v>72702</v>
       </c>
-      <c r="AK6" s="5" t="n">
+      <c r="AL6" s="5" t="n">
         <v>29.2</v>
       </c>
-      <c r="AL6" s="5" t="n">
+      <c r="AM6" s="5" t="n">
         <v>38.8</v>
       </c>
-      <c r="AM6" s="5" t="n">
+      <c r="AN6" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="AN6" s="5" t="n">
+      <c r="AO6" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="AO6" s="4" t="n">
+      <c r="AP6" s="4" t="n">
         <v>0.12</v>
       </c>
-      <c r="AP6" s="4" t="n">
+      <c r="AQ6" s="4" t="n">
         <v>0.562</v>
       </c>
-      <c r="AQ6" s="4" t="n">
+      <c r="AR6" s="4" t="n">
         <v>0.864</v>
       </c>
-      <c r="AR6" s="5" t="n">
+      <c r="AS6" s="5" t="n">
         <v>220</v>
       </c>
-      <c r="AS6" s="5" t="n">
+      <c r="AT6" s="5" t="n">
         <v>4417</v>
       </c>
-      <c r="AT6" s="5" t="n">
+      <c r="AU6" s="5" t="n">
         <v>24186.86</v>
       </c>
-      <c r="AU6" s="4" t="n">
+      <c r="AV6" s="4" t="n">
         <v>0.273</v>
       </c>
-      <c r="AV6" s="4" t="n">
+      <c r="AW6" s="4" t="n">
         <v>0.538</v>
       </c>
-      <c r="AW6" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="AX6" s="4" t="n">
+      <c r="AX6" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="AY6" s="4" t="n">
         <v>0.7231</v>
       </c>
-      <c r="AY6" s="4" t="n">
+      <c r="AZ6" s="4" t="n">
         <v>0.6189</v>
       </c>
-      <c r="AZ6" s="4" t="n">
+      <c r="BA6" s="4" t="n">
         <v>0.7325</v>
       </c>
-      <c r="BA6" s="5" t="n">
+      <c r="BB6" s="5" t="n">
         <v>186</v>
       </c>
-      <c r="BB6" s="4" t="n">
+      <c r="BC6" s="4" t="n">
         <v>-0.516234188182291</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D7" s="4" t="n">
         <v>0.289</v>
@@ -1790,124 +1812,127 @@
       <c r="R7" s="5" t="n">
         <v>13100</v>
       </c>
-      <c r="S7" s="4" t="n">
+      <c r="S7" s="5" t="n">
+        <v>33123</v>
+      </c>
+      <c r="T7" s="4" t="n">
         <v>0.018</v>
       </c>
-      <c r="T7" s="4" t="n">
+      <c r="U7" s="4" t="n">
         <v>0.276</v>
       </c>
-      <c r="U7" s="5" t="n">
+      <c r="V7" s="5" t="n">
         <v>187400</v>
       </c>
-      <c r="V7" s="5" t="n">
+      <c r="W7" s="5" t="n">
         <v>125141</v>
       </c>
-      <c r="W7" s="5" t="n">
+      <c r="X7" s="5" t="n">
         <v>0.59</v>
       </c>
-      <c r="X7" s="5" t="n">
+      <c r="Y7" s="5" t="n">
         <v>36480</v>
       </c>
-      <c r="Y7" s="5" t="n">
+      <c r="Z7" s="5" t="n">
         <v>5362</v>
       </c>
-      <c r="Z7" s="5" t="n">
+      <c r="AA7" s="5" t="n">
         <v>24.5</v>
       </c>
-      <c r="AA7" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="AB7" s="5" t="n">
+      <c r="AB7" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC7" s="5" t="n">
         <v>74990</v>
       </c>
-      <c r="AC7" s="5" t="n">
+      <c r="AD7" s="5" t="n">
         <v>45880</v>
       </c>
-      <c r="AD7" s="5" t="n">
+      <c r="AE7" s="5" t="n">
         <v>29780</v>
       </c>
-      <c r="AE7" s="5" t="n">
+      <c r="AF7" s="5" t="n">
         <v>158700</v>
       </c>
-      <c r="AF7" s="5" t="n">
+      <c r="AG7" s="5" t="n">
         <v>98750</v>
       </c>
-      <c r="AG7" s="5" t="n">
+      <c r="AH7" s="5" t="n">
         <v>62690</v>
       </c>
-      <c r="AH7" s="5" t="n">
+      <c r="AI7" s="5" t="n">
         <v>210</v>
       </c>
-      <c r="AI7" s="4" t="n">
+      <c r="AJ7" s="4" t="n">
         <v>0.588</v>
       </c>
-      <c r="AJ7" s="5" t="n">
+      <c r="AK7" s="5" t="n">
         <v>1809820</v>
       </c>
-      <c r="AK7" s="5" t="n">
+      <c r="AL7" s="5" t="n">
         <v>29.5</v>
       </c>
-      <c r="AL7" s="5" t="n">
+      <c r="AM7" s="5" t="n">
         <v>39</v>
       </c>
-      <c r="AM7" s="5" t="n">
+      <c r="AN7" s="5" t="n">
         <v>702</v>
       </c>
-      <c r="AN7" s="5" t="n">
+      <c r="AO7" s="5" t="n">
         <v>85</v>
       </c>
-      <c r="AO7" s="4" t="n">
+      <c r="AP7" s="4" t="n">
         <v>0.162</v>
       </c>
-      <c r="AP7" s="4" t="n">
+      <c r="AQ7" s="4" t="n">
         <v>0.369</v>
       </c>
-      <c r="AQ7" s="4" t="n">
+      <c r="AR7" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="AR7" s="5" t="n">
+      <c r="AS7" s="5" t="n">
         <v>434</v>
       </c>
-      <c r="AS7" s="5" t="n">
+      <c r="AT7" s="5" t="n">
         <v>5229</v>
       </c>
-      <c r="AT7" s="5" t="n">
+      <c r="AU7" s="5" t="n">
         <v>15209.61</v>
       </c>
-      <c r="AU7" s="4" t="n">
+      <c r="AV7" s="4" t="n">
         <v>0.298</v>
       </c>
-      <c r="AV7" s="4" t="n">
+      <c r="AW7" s="4" t="n">
         <v>0.538</v>
       </c>
-      <c r="AW7" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="AX7" s="4" t="n">
+      <c r="AX7" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="AY7" s="4" t="n">
         <v>0.7669</v>
       </c>
-      <c r="AY7" s="4" t="n">
+      <c r="AZ7" s="4" t="n">
         <v>0.656</v>
       </c>
-      <c r="AZ7" s="4" t="n">
+      <c r="BA7" s="4" t="n">
         <v>0.7817</v>
       </c>
-      <c r="BA7" s="5" t="n">
+      <c r="BB7" s="5" t="n">
         <v>408</v>
       </c>
-      <c r="BB7" s="4" t="n">
+      <c r="BC7" s="4" t="n">
         <v>-0.368102942649099</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D8" s="4" t="n">
         <v>0.13</v>
@@ -1954,124 +1979,127 @@
       <c r="R8" s="5" t="n">
         <v>4040</v>
       </c>
-      <c r="S8" s="4" t="n">
+      <c r="S8" s="5" t="n">
+        <v>19816</v>
+      </c>
+      <c r="T8" s="4" t="n">
         <v>0.096</v>
       </c>
-      <c r="T8" s="4" t="n">
+      <c r="U8" s="4" t="n">
         <v>0.292</v>
       </c>
-      <c r="U8" s="5" t="n">
+      <c r="V8" s="5" t="n">
         <v>19021100</v>
       </c>
-      <c r="V8" s="5" t="n">
+      <c r="W8" s="5" t="n">
         <v>1754992</v>
       </c>
-      <c r="W8" s="5" t="n">
+      <c r="X8" s="5" t="n">
         <v>0.43</v>
       </c>
-      <c r="X8" s="5" t="n">
+      <c r="Y8" s="5" t="n">
         <v>40180</v>
       </c>
-      <c r="Y8" s="5" t="n">
+      <c r="Z8" s="5" t="n">
         <v>18814</v>
       </c>
-      <c r="Z8" s="5" t="n">
+      <c r="AA8" s="5" t="n">
         <v>46.7</v>
       </c>
-      <c r="AA8" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="AB8" s="5" t="n">
+      <c r="AB8" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC8" s="5" t="n">
         <v>45620</v>
       </c>
-      <c r="AC8" s="5" t="n">
+      <c r="AD8" s="5" t="n">
         <v>33910</v>
       </c>
-      <c r="AD8" s="5" t="n">
+      <c r="AE8" s="5" t="n">
         <v>18960</v>
       </c>
-      <c r="AE8" s="5" t="n">
+      <c r="AF8" s="5" t="n">
         <v>107250</v>
       </c>
-      <c r="AF8" s="5" t="n">
+      <c r="AG8" s="5" t="n">
         <v>79050</v>
       </c>
-      <c r="AG8" s="5" t="n">
+      <c r="AH8" s="5" t="n">
         <v>44460</v>
       </c>
-      <c r="AH8" s="5" t="n">
+      <c r="AI8" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="AI8" s="4" t="n">
+      <c r="AJ8" s="4" t="n">
         <v>0.143</v>
       </c>
-      <c r="AJ8" s="5" t="n">
+      <c r="AK8" s="5" t="n">
         <v>149304</v>
       </c>
-      <c r="AK8" s="5" t="n">
+      <c r="AL8" s="5" t="n">
         <v>29.9</v>
       </c>
-      <c r="AL8" s="5" t="n">
+      <c r="AM8" s="5" t="n">
         <v>40.6</v>
       </c>
-      <c r="AM8" s="5" t="n">
+      <c r="AN8" s="5" t="n">
         <v>171</v>
       </c>
-      <c r="AN8" s="5" t="n">
+      <c r="AO8" s="5" t="n">
         <v>27</v>
       </c>
-      <c r="AO8" s="4" t="n">
+      <c r="AP8" s="4" t="n">
         <v>0.071</v>
       </c>
-      <c r="AP8" s="4" t="n">
+      <c r="AQ8" s="4" t="n">
         <v>0.548</v>
       </c>
-      <c r="AQ8" s="4" t="n">
+      <c r="AR8" s="4" t="n">
         <v>0.911</v>
       </c>
-      <c r="AR8" s="5" t="n">
+      <c r="AS8" s="5" t="n">
         <v>175</v>
       </c>
-      <c r="AS8" s="5" t="n">
+      <c r="AT8" s="5" t="n">
         <v>6303</v>
       </c>
-      <c r="AT8" s="5" t="n">
+      <c r="AU8" s="5" t="n">
         <v>77490.24</v>
       </c>
-      <c r="AU8" s="4" t="n">
+      <c r="AV8" s="4" t="n">
         <v>0.465</v>
       </c>
-      <c r="AV8" s="4" t="n">
+      <c r="AW8" s="4" t="n">
         <v>0.538</v>
       </c>
-      <c r="AW8" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="AX8" s="4" t="n">
+      <c r="AX8" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="AY8" s="4" t="n">
         <v>0.7894</v>
       </c>
-      <c r="AY8" s="4" t="n">
+      <c r="AZ8" s="4" t="n">
         <v>0.6734</v>
       </c>
-      <c r="AZ8" s="4" t="n">
+      <c r="BA8" s="4" t="n">
         <v>0.8204</v>
       </c>
-      <c r="BA8" s="5" t="n">
+      <c r="BB8" s="5" t="n">
         <v>1159</v>
       </c>
-      <c r="BB8" s="4" t="n">
+      <c r="BC8" s="4" t="n">
         <v>-0.351294943553743</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D9" s="4" t="n">
         <v>0.256</v>
@@ -2118,124 +2146,127 @@
       <c r="R9" s="5" t="n">
         <v>4317</v>
       </c>
-      <c r="S9" s="4" t="n">
+      <c r="S9" s="5" t="n">
+        <v>16290</v>
+      </c>
+      <c r="T9" s="4" t="n">
         <v>0.06</v>
       </c>
-      <c r="T9" s="4" t="n">
+      <c r="U9" s="4" t="n">
         <v>0.267</v>
       </c>
-      <c r="U9" s="5" t="n">
+      <c r="V9" s="5" t="n">
         <v>2129700</v>
       </c>
-      <c r="V9" s="5" t="n">
+      <c r="W9" s="5" t="n">
         <v>334743</v>
       </c>
-      <c r="W9" s="5" t="n">
+      <c r="X9" s="5" t="n">
         <v>0.51</v>
       </c>
-      <c r="X9" s="5" t="n">
+      <c r="Y9" s="5" t="n">
         <v>22670</v>
       </c>
-      <c r="Y9" s="5" t="n">
+      <c r="Z9" s="5" t="n">
         <v>8344</v>
       </c>
-      <c r="Z9" s="5" t="n">
+      <c r="AA9" s="5" t="n">
         <v>37.6</v>
       </c>
-      <c r="AA9" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="AB9" s="5" t="n">
+      <c r="AB9" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC9" s="5" t="n">
         <v>55040</v>
       </c>
-      <c r="AC9" s="5" t="n">
+      <c r="AD9" s="5" t="n">
         <v>37040</v>
       </c>
-      <c r="AD9" s="5" t="n">
+      <c r="AE9" s="5" t="n">
         <v>22970</v>
       </c>
-      <c r="AE9" s="5" t="n">
+      <c r="AF9" s="5" t="n">
         <v>98500</v>
       </c>
-      <c r="AF9" s="5" t="n">
+      <c r="AG9" s="5" t="n">
         <v>65950</v>
       </c>
-      <c r="AG9" s="5" t="n">
+      <c r="AH9" s="5" t="n">
         <v>41840</v>
       </c>
-      <c r="AH9" s="5" t="n">
+      <c r="AI9" s="5" t="n">
         <v>27</v>
       </c>
-      <c r="AI9" s="4" t="n">
+      <c r="AJ9" s="4" t="n">
         <v>0.229</v>
       </c>
-      <c r="AJ9" s="5" t="n">
+      <c r="AK9" s="5" t="n">
         <v>234485</v>
       </c>
-      <c r="AK9" s="5" t="n">
+      <c r="AL9" s="5" t="n">
         <v>30.8</v>
       </c>
-      <c r="AL9" s="5" t="n">
+      <c r="AM9" s="5" t="n">
         <v>35.8</v>
       </c>
-      <c r="AM9" s="5" t="n">
+      <c r="AN9" s="5" t="n">
         <v>182</v>
       </c>
-      <c r="AN9" s="5" t="n">
+      <c r="AO9" s="5" t="n">
         <v>21</v>
       </c>
-      <c r="AO9" s="4" t="n">
+      <c r="AP9" s="4" t="n">
         <v>0.147</v>
       </c>
-      <c r="AP9" s="4" t="n">
+      <c r="AQ9" s="4" t="n">
         <v>0.394</v>
       </c>
-      <c r="AQ9" s="4" t="n">
+      <c r="AR9" s="4" t="n">
         <v>0.807</v>
       </c>
-      <c r="AR9" s="5" t="n">
+      <c r="AS9" s="5" t="n">
         <v>380</v>
       </c>
-      <c r="AS9" s="5" t="n">
+      <c r="AT9" s="5" t="n">
         <v>11568</v>
       </c>
-      <c r="AT9" s="5" t="n">
+      <c r="AU9" s="5" t="n">
         <v>79242.19</v>
       </c>
-      <c r="AU9" s="4" t="n">
+      <c r="AV9" s="4" t="n">
         <v>0.521</v>
       </c>
-      <c r="AV9" s="4" t="n">
+      <c r="AW9" s="4" t="n">
         <v>0.538</v>
       </c>
-      <c r="AW9" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="AX9" s="4" t="n">
+      <c r="AX9" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="AY9" s="4" t="n">
         <v>0.8389</v>
       </c>
-      <c r="AY9" s="4" t="n">
+      <c r="AZ9" s="4" t="n">
         <v>0.7064</v>
       </c>
-      <c r="AZ9" s="4" t="n">
+      <c r="BA9" s="4" t="n">
         <v>0.8452</v>
       </c>
-      <c r="BA9" s="5" t="n">
+      <c r="BB9" s="5" t="n">
         <v>609</v>
       </c>
-      <c r="BB9" s="4" t="n">
+      <c r="BC9" s="4" t="n">
         <v>-0.470422736215456</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D10" s="4" t="n">
         <v>0.171</v>
@@ -2282,122 +2313,125 @@
       <c r="R10" s="5" t="n">
         <v>3667</v>
       </c>
-      <c r="S10" s="4" t="n">
+      <c r="S10" s="5" t="n">
+        <v>17003</v>
+      </c>
+      <c r="T10" s="4" t="n">
         <v>0.051</v>
       </c>
-      <c r="T10" s="4" t="n">
+      <c r="U10" s="4" t="n">
         <v>0.258</v>
       </c>
-      <c r="U10" s="5" t="n">
+      <c r="V10" s="5" t="n">
         <v>60497100</v>
       </c>
-      <c r="V10" s="5" t="n">
+      <c r="W10" s="5" t="n">
         <v>10852073</v>
       </c>
-      <c r="W10" s="5"/>
-      <c r="X10" s="5" t="n">
+      <c r="X10" s="5"/>
+      <c r="Y10" s="5" t="n">
         <v>27160</v>
       </c>
-      <c r="Y10" s="5" t="n">
+      <c r="Z10" s="5" t="n">
         <v>15170</v>
       </c>
-      <c r="Z10" s="5" t="n">
+      <c r="AA10" s="5" t="n">
         <v>2309.4</v>
       </c>
-      <c r="AA10" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="AB10" s="5" t="n">
+      <c r="AB10" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="AC10" s="5" t="n">
         <v>34000</v>
       </c>
-      <c r="AC10" s="5" t="n">
+      <c r="AD10" s="5" t="n">
         <v>32790</v>
       </c>
-      <c r="AD10" s="5" t="n">
+      <c r="AE10" s="5" t="n">
         <v>14880</v>
       </c>
-      <c r="AE10" s="5" t="n">
+      <c r="AF10" s="5" t="n">
         <v>64850</v>
       </c>
-      <c r="AF10" s="5" t="n">
+      <c r="AG10" s="5" t="n">
         <v>58630</v>
       </c>
-      <c r="AG10" s="5" t="n">
+      <c r="AH10" s="5" t="n">
         <v>28640</v>
       </c>
-      <c r="AH10" s="5" t="n">
+      <c r="AI10" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="AI10" s="4" t="n">
+      <c r="AJ10" s="4" t="n">
         <v>0.069</v>
       </c>
-      <c r="AJ10" s="5" t="n">
+      <c r="AK10" s="5" t="n">
         <v>55993</v>
       </c>
-      <c r="AK10" s="5" t="n">
+      <c r="AL10" s="5" t="n">
         <v>29</v>
       </c>
-      <c r="AL10" s="5" t="n">
+      <c r="AM10" s="5" t="n">
         <v>40</v>
       </c>
-      <c r="AM10" s="5" t="n">
+      <c r="AN10" s="5" t="n">
         <v>56</v>
       </c>
-      <c r="AN10" s="5" t="n">
+      <c r="AO10" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="AO10" s="4" t="n">
+      <c r="AP10" s="4" t="n">
         <v>0.119</v>
       </c>
-      <c r="AP10" s="4" t="n">
+      <c r="AQ10" s="4" t="n">
         <v>0.488</v>
       </c>
-      <c r="AQ10" s="4" t="n">
+      <c r="AR10" s="4" t="n">
         <v>0.87</v>
       </c>
-      <c r="AR10" s="5" t="n">
+      <c r="AS10" s="5" t="n">
         <v>639</v>
       </c>
-      <c r="AS10" s="5" t="n">
+      <c r="AT10" s="5" t="n">
         <v>24460</v>
       </c>
-      <c r="AT10" s="5" t="n">
+      <c r="AU10" s="5" t="n">
         <v>196115.77</v>
       </c>
-      <c r="AU10" s="4" t="n">
+      <c r="AV10" s="4" t="n">
         <v>0.432</v>
       </c>
-      <c r="AV10" s="4" t="n">
+      <c r="AW10" s="4" t="n">
         <v>0.538</v>
       </c>
-      <c r="AW10" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="AX10" s="4" t="n">
+      <c r="AX10" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="AY10" s="4" t="n">
         <v>0.781</v>
       </c>
-      <c r="AY10" s="4" t="n">
+      <c r="AZ10" s="4" t="n">
         <v>0.6628</v>
       </c>
-      <c r="AZ10" s="4" t="n">
+      <c r="BA10" s="4" t="n">
         <v>0.8156</v>
       </c>
-      <c r="BA10" s="5" t="n">
+      <c r="BB10" s="5" t="n">
         <v>439</v>
       </c>
-      <c r="BB10" s="4" t="n">
+      <c r="BC10" s="4" t="n">
         <v>-0.424527305376571</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D11" s="4" t="n">
         <v>0.181</v>
@@ -2444,122 +2478,125 @@
       <c r="R11" s="5" t="n">
         <v>9893</v>
       </c>
-      <c r="S11" s="4" t="n">
+      <c r="S11" s="5" t="n">
+        <v>40964</v>
+      </c>
+      <c r="T11" s="4" t="n">
         <v>0.027</v>
       </c>
-      <c r="T11" s="4" t="n">
+      <c r="U11" s="4" t="n">
         <v>0.244</v>
       </c>
-      <c r="U11" s="5" t="n">
+      <c r="V11" s="5" t="n">
         <v>42378000</v>
       </c>
-      <c r="V11" s="5" t="n">
+      <c r="W11" s="5" t="n">
         <v>904304</v>
       </c>
-      <c r="W11" s="5"/>
-      <c r="X11" s="5" t="n">
+      <c r="X11" s="5"/>
+      <c r="Y11" s="5" t="n">
         <v>63650</v>
       </c>
-      <c r="Y11" s="5" t="n">
+      <c r="Z11" s="5" t="n">
         <v>14412</v>
       </c>
-      <c r="Z11" s="5" t="n">
+      <c r="AA11" s="5" t="n">
         <v>201.1</v>
       </c>
-      <c r="AA11" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="AB11" s="5" t="n">
+      <c r="AB11" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="AC11" s="5" t="n">
         <v>61540</v>
       </c>
-      <c r="AC11" s="5" t="n">
+      <c r="AD11" s="5" t="n">
         <v>49440</v>
       </c>
-      <c r="AD11" s="5" t="n">
+      <c r="AE11" s="5" t="n">
         <v>26410</v>
       </c>
-      <c r="AE11" s="5" t="n">
+      <c r="AF11" s="5" t="n">
         <v>129780</v>
       </c>
-      <c r="AF11" s="5" t="n">
+      <c r="AG11" s="5" t="n">
         <v>100590</v>
       </c>
-      <c r="AG11" s="5" t="n">
+      <c r="AH11" s="5" t="n">
         <v>56690</v>
       </c>
-      <c r="AH11" s="5" t="n">
+      <c r="AI11" s="5" t="n">
         <v>66</v>
       </c>
-      <c r="AI11" s="4" t="n">
+      <c r="AJ11" s="4" t="n">
         <v>0.247</v>
       </c>
-      <c r="AJ11" s="5" t="n">
+      <c r="AK11" s="5" t="n">
         <v>571483</v>
       </c>
-      <c r="AK11" s="5" t="n">
+      <c r="AL11" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="AL11" s="5" t="n">
+      <c r="AM11" s="5" t="n">
         <v>40.5</v>
       </c>
-      <c r="AM11" s="5" t="n">
+      <c r="AN11" s="5" t="n">
         <v>642</v>
       </c>
-      <c r="AN11" s="5" t="n">
+      <c r="AO11" s="5" t="n">
         <v>51</v>
       </c>
-      <c r="AO11" s="4" t="n">
+      <c r="AP11" s="4" t="n">
         <v>0.146</v>
       </c>
-      <c r="AP11" s="4" t="n">
+      <c r="AQ11" s="4" t="n">
         <v>0.447</v>
       </c>
-      <c r="AQ11" s="4" t="n">
+      <c r="AR11" s="4" t="n">
         <v>0.846</v>
       </c>
-      <c r="AR11" s="5" t="n">
+      <c r="AS11" s="5" t="n">
         <v>819</v>
       </c>
-      <c r="AS11" s="5" t="n">
+      <c r="AT11" s="5" t="n">
         <v>22334</v>
       </c>
-      <c r="AT11" s="5" t="n">
+      <c r="AU11" s="5" t="n">
         <v>151848.16</v>
       </c>
-      <c r="AU11" s="4" t="n">
+      <c r="AV11" s="4" t="n">
         <v>0.41</v>
       </c>
-      <c r="AV11" s="4" t="n">
+      <c r="AW11" s="4" t="n">
         <v>0.538</v>
       </c>
-      <c r="AW11" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="AX11" s="4" t="n">
+      <c r="AX11" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="AY11" s="4" t="n">
         <v>0.767</v>
       </c>
-      <c r="AY11" s="4" t="n">
+      <c r="AZ11" s="4" t="n">
         <v>0.6453</v>
       </c>
-      <c r="AZ11" s="4" t="n">
+      <c r="BA11" s="4" t="n">
         <v>0.7837</v>
       </c>
-      <c r="BA11" s="5" t="n">
+      <c r="BB11" s="5" t="n">
         <v>2364</v>
       </c>
-      <c r="BB11" s="4" t="n">
+      <c r="BC11" s="4" t="n">
         <v>-0.614607629122389</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D12" s="4" t="n">
         <v>0.278</v>
@@ -2606,122 +2643,125 @@
       <c r="R12" s="5" t="n">
         <v>8844</v>
       </c>
-      <c r="S12" s="4" t="n">
+      <c r="S12" s="5" t="n">
+        <v>29209</v>
+      </c>
+      <c r="T12" s="4" t="n">
         <v>0.018</v>
       </c>
-      <c r="T12" s="4" t="n">
+      <c r="U12" s="4" t="n">
         <v>0.242</v>
       </c>
-      <c r="U12" s="5" t="n">
+      <c r="V12" s="5" t="n">
         <v>25081500</v>
       </c>
-      <c r="V12" s="5" t="n">
+      <c r="W12" s="5" t="n">
         <v>1639888</v>
       </c>
-      <c r="W12" s="5"/>
-      <c r="X12" s="5" t="n">
+      <c r="X12" s="5"/>
+      <c r="Y12" s="5" t="n">
         <v>55670</v>
       </c>
-      <c r="Y12" s="5" t="n">
+      <c r="Z12" s="5" t="n">
         <v>10287</v>
       </c>
-      <c r="Z12" s="5" t="n">
+      <c r="AA12" s="5" t="n">
         <v>1063.3</v>
       </c>
-      <c r="AA12" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="AB12" s="5" t="n">
+      <c r="AB12" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="AC12" s="5" t="n">
         <v>52650</v>
       </c>
-      <c r="AC12" s="5" t="n">
+      <c r="AD12" s="5" t="n">
         <v>41700</v>
       </c>
-      <c r="AD12" s="5" t="n">
+      <c r="AE12" s="5" t="n">
         <v>23700</v>
       </c>
-      <c r="AE12" s="5" t="n">
+      <c r="AF12" s="5" t="n">
         <v>96590</v>
       </c>
-      <c r="AF12" s="5" t="n">
+      <c r="AG12" s="5" t="n">
         <v>73700</v>
       </c>
-      <c r="AG12" s="5" t="n">
+      <c r="AH12" s="5" t="n">
         <v>44330</v>
       </c>
-      <c r="AH12" s="5" t="n">
+      <c r="AI12" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="AI12" s="4" t="n">
+      <c r="AJ12" s="4" t="n">
         <v>0.004</v>
       </c>
-      <c r="AJ12" s="5" t="n">
+      <c r="AK12" s="5" t="n">
         <v>7530</v>
       </c>
-      <c r="AK12" s="5" t="n">
+      <c r="AL12" s="5" t="n">
         <v>27.4</v>
       </c>
-      <c r="AL12" s="5" t="n">
+      <c r="AM12" s="5" t="n">
         <v>37.3</v>
-      </c>
-      <c r="AM12" s="5" t="n">
-        <v>0</v>
       </c>
       <c r="AN12" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AO12" s="4" t="n">
+      <c r="AO12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP12" s="4" t="n">
         <v>0.172</v>
       </c>
-      <c r="AP12" s="4" t="n">
+      <c r="AQ12" s="4" t="n">
         <v>0.527</v>
       </c>
-      <c r="AQ12" s="4" t="n">
+      <c r="AR12" s="4" t="n">
         <v>0.842</v>
       </c>
-      <c r="AR12" s="5" t="n">
+      <c r="AS12" s="5" t="n">
         <v>1092</v>
       </c>
-      <c r="AS12" s="5" t="n">
+      <c r="AT12" s="5" t="n">
         <v>27623</v>
       </c>
-      <c r="AT12" s="5" t="n">
+      <c r="AU12" s="5" t="n">
         <v>172478.21</v>
       </c>
-      <c r="AU12" s="4" t="n">
+      <c r="AV12" s="4" t="n">
         <v>0.326</v>
       </c>
-      <c r="AV12" s="4" t="n">
+      <c r="AW12" s="4" t="n">
         <v>0.538</v>
       </c>
-      <c r="AW12" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="AX12" s="4" t="n">
+      <c r="AX12" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="AY12" s="4" t="n">
         <v>0.7527</v>
       </c>
-      <c r="AY12" s="4" t="n">
+      <c r="AZ12" s="4" t="n">
         <v>0.6454</v>
       </c>
-      <c r="AZ12" s="4" t="n">
+      <c r="BA12" s="4" t="n">
         <v>0.7656</v>
       </c>
-      <c r="BA12" s="5" t="n">
+      <c r="BB12" s="5" t="n">
         <v>443</v>
       </c>
-      <c r="BB12" s="4" t="n">
+      <c r="BC12" s="4" t="n">
         <v>-0.498492545506827</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D13" s="4" t="n">
         <v>0.184</v>
@@ -2768,122 +2808,125 @@
       <c r="R13" s="5" t="n">
         <v>2734</v>
       </c>
-      <c r="S13" s="4" t="n">
+      <c r="S13" s="5" t="n">
+        <v>9491</v>
+      </c>
+      <c r="T13" s="4" t="n">
         <v>0.06</v>
       </c>
-      <c r="T13" s="4" t="n">
+      <c r="U13" s="4" t="n">
         <v>0.327</v>
       </c>
-      <c r="U13" s="5" t="n">
+      <c r="V13" s="5" t="n">
         <v>28151200</v>
       </c>
-      <c r="V13" s="5" t="n">
+      <c r="W13" s="5" t="n">
         <v>1220687</v>
       </c>
-      <c r="W13" s="5"/>
-      <c r="X13" s="5" t="n">
+      <c r="X13" s="5"/>
+      <c r="Y13" s="5" t="n">
         <v>14430</v>
       </c>
-      <c r="Y13" s="5" t="n">
+      <c r="Z13" s="5" t="n">
         <v>4606</v>
       </c>
-      <c r="Z13" s="5" t="n">
+      <c r="AA13" s="5" t="n">
         <v>60.7</v>
       </c>
-      <c r="AA13" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="AB13" s="5" t="n">
+      <c r="AB13" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="AC13" s="5" t="n">
         <v>41670</v>
       </c>
-      <c r="AC13" s="5" t="n">
+      <c r="AD13" s="5" t="n">
         <v>31200</v>
       </c>
-      <c r="AD13" s="5" t="n">
+      <c r="AE13" s="5" t="n">
         <v>18430</v>
       </c>
-      <c r="AE13" s="5" t="n">
+      <c r="AF13" s="5" t="n">
         <v>62720</v>
       </c>
-      <c r="AF13" s="5" t="n">
+      <c r="AG13" s="5" t="n">
         <v>48310</v>
       </c>
-      <c r="AG13" s="5" t="n">
+      <c r="AH13" s="5" t="n">
         <v>28190</v>
       </c>
-      <c r="AH13" s="5" t="n">
+      <c r="AI13" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="AI13" s="4" t="n">
+      <c r="AJ13" s="4" t="n">
         <v>0.026</v>
       </c>
-      <c r="AJ13" s="5" t="n">
+      <c r="AK13" s="5" t="n">
         <v>18073</v>
       </c>
-      <c r="AK13" s="5" t="n">
+      <c r="AL13" s="5" t="n">
         <v>28.7</v>
       </c>
-      <c r="AL13" s="5" t="n">
+      <c r="AM13" s="5" t="n">
         <v>39.6</v>
       </c>
-      <c r="AM13" s="5" t="n">
+      <c r="AN13" s="5" t="n">
         <v>31</v>
       </c>
-      <c r="AN13" s="5" t="n">
+      <c r="AO13" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="AO13" s="4" t="n">
+      <c r="AP13" s="4" t="n">
         <v>0.068</v>
       </c>
-      <c r="AP13" s="4" t="n">
+      <c r="AQ13" s="4" t="n">
         <v>0.675</v>
       </c>
-      <c r="AQ13" s="4" t="n">
+      <c r="AR13" s="4" t="n">
         <v>0.94</v>
       </c>
-      <c r="AR13" s="5" t="n">
+      <c r="AS13" s="5" t="n">
         <v>146</v>
       </c>
-      <c r="AS13" s="5" t="n">
+      <c r="AT13" s="5" t="n">
         <v>4794</v>
       </c>
-      <c r="AT13" s="5" t="n">
+      <c r="AU13" s="5" t="n">
         <v>50765.35</v>
-      </c>
-      <c r="AU13" s="4" t="n">
-        <v>0.538</v>
       </c>
       <c r="AV13" s="4" t="n">
         <v>0.538</v>
       </c>
-      <c r="AW13" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="AX13" s="4" t="n">
+      <c r="AW13" s="4" t="n">
+        <v>0.538</v>
+      </c>
+      <c r="AX13" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="AY13" s="4" t="n">
         <v>0.7352</v>
       </c>
-      <c r="AY13" s="4" t="n">
+      <c r="AZ13" s="4" t="n">
         <v>0.616</v>
       </c>
-      <c r="AZ13" s="4" t="n">
+      <c r="BA13" s="4" t="n">
         <v>0.7441</v>
       </c>
-      <c r="BA13" s="5" t="n">
+      <c r="BB13" s="5" t="n">
         <v>197</v>
       </c>
-      <c r="BB13" s="4" t="n">
+      <c r="BC13" s="4" t="n">
         <v>-0.694391871700369</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D14" s="4" t="n">
         <v>0.109</v>
@@ -2930,122 +2973,125 @@
       <c r="R14" s="5" t="n">
         <v>4884</v>
       </c>
-      <c r="S14" s="4" t="n">
+      <c r="S14" s="5" t="n">
+        <v>18672</v>
+      </c>
+      <c r="T14" s="4" t="n">
         <v>0.046</v>
       </c>
-      <c r="T14" s="4" t="n">
+      <c r="U14" s="4" t="n">
         <v>0.286</v>
       </c>
-      <c r="U14" s="5" t="n">
+      <c r="V14" s="5" t="n">
         <v>82376900</v>
       </c>
-      <c r="V14" s="5" t="n">
+      <c r="W14" s="5" t="n">
         <v>1541121</v>
       </c>
-      <c r="W14" s="5"/>
-      <c r="X14" s="5" t="n">
+      <c r="X14" s="5"/>
+      <c r="Y14" s="5" t="n">
         <v>44270</v>
       </c>
-      <c r="Y14" s="5" t="n">
+      <c r="Z14" s="5" t="n">
         <v>20519</v>
       </c>
-      <c r="Z14" s="5" t="n">
+      <c r="AA14" s="5" t="n">
         <v>69.2</v>
       </c>
-      <c r="AA14" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="AB14" s="5" t="n">
+      <c r="AB14" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="AC14" s="5" t="n">
         <v>64400</v>
       </c>
-      <c r="AC14" s="5" t="n">
+      <c r="AD14" s="5" t="n">
         <v>76070</v>
       </c>
-      <c r="AD14" s="5" t="n">
+      <c r="AE14" s="5" t="n">
         <v>29440</v>
       </c>
-      <c r="AE14" s="5" t="n">
+      <c r="AF14" s="5" t="n">
         <v>152940</v>
       </c>
-      <c r="AF14" s="5" t="n">
+      <c r="AG14" s="5" t="n">
         <v>139510</v>
       </c>
-      <c r="AG14" s="5" t="n">
+      <c r="AH14" s="5" t="n">
         <v>67890</v>
       </c>
-      <c r="AH14" s="5" t="n">
+      <c r="AI14" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="AI14" s="4" t="n">
+      <c r="AJ14" s="4" t="n">
         <v>0.173</v>
       </c>
-      <c r="AJ14" s="5" t="n">
+      <c r="AK14" s="5" t="n">
         <v>191487</v>
       </c>
-      <c r="AK14" s="5" t="n">
+      <c r="AL14" s="5" t="n">
         <v>30.2</v>
       </c>
-      <c r="AL14" s="5" t="n">
+      <c r="AM14" s="5" t="n">
         <v>40.4</v>
       </c>
-      <c r="AM14" s="5" t="n">
+      <c r="AN14" s="5" t="n">
         <v>275</v>
       </c>
-      <c r="AN14" s="5" t="n">
+      <c r="AO14" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="AO14" s="4" t="n">
+      <c r="AP14" s="4" t="n">
         <v>0.069</v>
       </c>
-      <c r="AP14" s="4" t="n">
+      <c r="AQ14" s="4" t="n">
         <v>0.736</v>
       </c>
-      <c r="AQ14" s="4" t="n">
+      <c r="AR14" s="4" t="n">
         <v>0.953</v>
       </c>
-      <c r="AR14" s="5" t="n">
+      <c r="AS14" s="5" t="n">
         <v>254</v>
       </c>
-      <c r="AS14" s="5" t="n">
+      <c r="AT14" s="5" t="n">
         <v>7081</v>
       </c>
-      <c r="AT14" s="5" t="n">
+      <c r="AU14" s="5" t="n">
         <v>72612.65</v>
       </c>
-      <c r="AU14" s="4" t="n">
+      <c r="AV14" s="4" t="n">
         <v>0.404</v>
       </c>
-      <c r="AV14" s="4" t="n">
+      <c r="AW14" s="4" t="n">
         <v>0.538</v>
       </c>
-      <c r="AW14" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="AX14" s="4" t="n">
+      <c r="AX14" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="AY14" s="4" t="n">
         <v>0.7324</v>
       </c>
-      <c r="AY14" s="4" t="n">
+      <c r="AZ14" s="4" t="n">
         <v>0.6124</v>
       </c>
-      <c r="AZ14" s="4" t="n">
+      <c r="BA14" s="4" t="n">
         <v>0.7518</v>
       </c>
-      <c r="BA14" s="5" t="n">
+      <c r="BB14" s="5" t="n">
         <v>938</v>
       </c>
-      <c r="BB14" s="4" t="n">
+      <c r="BC14" s="4" t="n">
         <v>-0.30594391465977</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D15" s="4" t="n">
         <v>0.142</v>
@@ -3092,122 +3138,125 @@
       <c r="R15" s="5" t="n">
         <v>2220</v>
       </c>
-      <c r="S15" s="4" t="n">
+      <c r="S15" s="5" t="n">
+        <v>7264</v>
+      </c>
+      <c r="T15" s="4" t="n">
         <v>0.028</v>
       </c>
-      <c r="T15" s="4" t="n">
+      <c r="U15" s="4" t="n">
         <v>0.247</v>
       </c>
-      <c r="U15" s="5" t="n">
+      <c r="V15" s="5" t="n">
         <v>41935700</v>
       </c>
-      <c r="V15" s="5" t="n">
+      <c r="W15" s="5" t="n">
         <v>1029442</v>
       </c>
-      <c r="W15" s="5"/>
-      <c r="X15" s="5" t="n">
+      <c r="X15" s="5"/>
+      <c r="Y15" s="5" t="n">
         <v>16200</v>
       </c>
-      <c r="Y15" s="5" t="n">
+      <c r="Z15" s="5" t="n">
         <v>6991</v>
       </c>
-      <c r="Z15" s="5" t="n">
+      <c r="AA15" s="5" t="n">
         <v>4613.7</v>
       </c>
-      <c r="AA15" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="AB15" s="5" t="n">
+      <c r="AB15" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="AC15" s="5" t="n">
         <v>21430</v>
       </c>
-      <c r="AC15" s="5" t="n">
+      <c r="AD15" s="5" t="n">
         <v>21120</v>
       </c>
-      <c r="AD15" s="5" t="n">
+      <c r="AE15" s="5" t="n">
         <v>9860</v>
       </c>
-      <c r="AE15" s="5" t="n">
+      <c r="AF15" s="5" t="n">
         <v>34430</v>
       </c>
-      <c r="AF15" s="5" t="n">
+      <c r="AG15" s="5" t="n">
         <v>33100</v>
       </c>
-      <c r="AG15" s="5" t="n">
+      <c r="AH15" s="5" t="n">
         <v>16090</v>
       </c>
-      <c r="AH15" s="5" t="n">
+      <c r="AI15" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AI15" s="4" t="n">
+      <c r="AJ15" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AJ15" s="5" t="n">
+      <c r="AK15" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AK15" s="5" t="n">
+      <c r="AL15" s="5" t="n">
         <v>27.3</v>
       </c>
-      <c r="AL15" s="5" t="n">
+      <c r="AM15" s="5" t="n">
         <v>35.6</v>
-      </c>
-      <c r="AM15" s="5" t="n">
-        <v>0</v>
       </c>
       <c r="AN15" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AO15" s="4" t="n">
+      <c r="AO15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP15" s="4" t="n">
         <v>0.139</v>
       </c>
-      <c r="AP15" s="4" t="n">
+      <c r="AQ15" s="4" t="n">
         <v>0.555</v>
       </c>
-      <c r="AQ15" s="4" t="n">
+      <c r="AR15" s="4" t="n">
         <v>0.9</v>
       </c>
-      <c r="AR15" s="5" t="n">
+      <c r="AS15" s="5" t="n">
         <v>402</v>
       </c>
-      <c r="AS15" s="5" t="n">
+      <c r="AT15" s="5" t="n">
         <v>19698</v>
       </c>
-      <c r="AT15" s="5" t="n">
+      <c r="AU15" s="5" t="n">
         <v>157330.25</v>
       </c>
-      <c r="AU15" s="4" t="n">
+      <c r="AV15" s="4" t="n">
         <v>0.507</v>
       </c>
-      <c r="AV15" s="4" t="n">
+      <c r="AW15" s="4" t="n">
         <v>0.538</v>
       </c>
-      <c r="AW15" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="AX15" s="4" t="n">
+      <c r="AX15" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="AY15" s="4" t="n">
         <v>0.7613</v>
       </c>
-      <c r="AY15" s="4" t="n">
+      <c r="AZ15" s="4" t="n">
         <v>0.6376</v>
       </c>
-      <c r="AZ15" s="4" t="n">
+      <c r="BA15" s="4" t="n">
         <v>0.7652</v>
       </c>
-      <c r="BA15" s="5" t="n">
+      <c r="BB15" s="5" t="n">
         <v>256</v>
       </c>
-      <c r="BB15" s="4" t="n">
+      <c r="BC15" s="4" t="n">
         <v>-0.334270064301024</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D16" s="4" t="n">
         <v>0.162</v>
@@ -3254,122 +3303,125 @@
       <c r="R16" s="5" t="n">
         <v>4350</v>
       </c>
-      <c r="S16" s="4" t="n">
+      <c r="S16" s="5" t="n">
+        <v>24592</v>
+      </c>
+      <c r="T16" s="4" t="n">
         <v>0.029</v>
       </c>
-      <c r="T16" s="4" t="n">
+      <c r="U16" s="4" t="n">
         <v>0.256</v>
       </c>
-      <c r="U16" s="5" t="n">
+      <c r="V16" s="5" t="n">
         <v>18533700</v>
       </c>
-      <c r="V16" s="5" t="n">
+      <c r="W16" s="5" t="n">
         <v>365158</v>
       </c>
-      <c r="W16" s="5"/>
-      <c r="X16" s="5" t="n">
+      <c r="X16" s="5"/>
+      <c r="Y16" s="5" t="n">
         <v>25360</v>
       </c>
-      <c r="Y16" s="5" t="n">
+      <c r="Z16" s="5" t="n">
         <v>6457</v>
       </c>
-      <c r="Z16" s="5" t="n">
+      <c r="AA16" s="5" t="n">
         <v>66.4</v>
       </c>
-      <c r="AA16" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="AB16" s="5" t="n">
+      <c r="AB16" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="AC16" s="5" t="n">
         <v>29940</v>
       </c>
-      <c r="AC16" s="5" t="n">
+      <c r="AD16" s="5" t="n">
         <v>26240</v>
       </c>
-      <c r="AD16" s="5" t="n">
+      <c r="AE16" s="5" t="n">
         <v>13070</v>
       </c>
-      <c r="AE16" s="5" t="n">
+      <c r="AF16" s="5" t="n">
         <v>57820</v>
       </c>
-      <c r="AF16" s="5" t="n">
+      <c r="AG16" s="5" t="n">
         <v>45600</v>
       </c>
-      <c r="AG16" s="5" t="n">
+      <c r="AH16" s="5" t="n">
         <v>25480</v>
       </c>
-      <c r="AH16" s="5" t="n">
+      <c r="AI16" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="AI16" s="4" t="n">
+      <c r="AJ16" s="4" t="n">
         <v>0.065</v>
       </c>
-      <c r="AJ16" s="5" t="n">
+      <c r="AK16" s="5" t="n">
         <v>63774</v>
       </c>
-      <c r="AK16" s="5" t="n">
+      <c r="AL16" s="5" t="n">
         <v>28.7</v>
       </c>
-      <c r="AL16" s="5" t="n">
+      <c r="AM16" s="5" t="n">
         <v>38.4</v>
       </c>
-      <c r="AM16" s="5" t="n">
+      <c r="AN16" s="5" t="n">
         <v>68</v>
       </c>
-      <c r="AN16" s="5" t="n">
+      <c r="AO16" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="AO16" s="4" t="n">
+      <c r="AP16" s="4" t="n">
         <v>0.137</v>
       </c>
-      <c r="AP16" s="4" t="n">
+      <c r="AQ16" s="4" t="n">
         <v>0.373</v>
       </c>
-      <c r="AQ16" s="4" t="n">
+      <c r="AR16" s="4" t="n">
         <v>0.828</v>
       </c>
-      <c r="AR16" s="5" t="n">
+      <c r="AS16" s="5" t="n">
         <v>312</v>
       </c>
-      <c r="AS16" s="5" t="n">
+      <c r="AT16" s="5" t="n">
         <v>10181</v>
       </c>
-      <c r="AT16" s="5" t="n">
+      <c r="AU16" s="5" t="n">
         <v>60764.87</v>
       </c>
-      <c r="AU16" s="4" t="n">
+      <c r="AV16" s="4" t="n">
         <v>0.519</v>
       </c>
-      <c r="AV16" s="4" t="n">
+      <c r="AW16" s="4" t="n">
         <v>0.538</v>
       </c>
-      <c r="AW16" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="AX16" s="4" t="n">
+      <c r="AX16" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="AY16" s="4" t="n">
         <v>0.7842</v>
       </c>
-      <c r="AY16" s="4" t="n">
+      <c r="AZ16" s="4" t="n">
         <v>0.6613</v>
       </c>
-      <c r="AZ16" s="4" t="n">
+      <c r="BA16" s="4" t="n">
         <v>0.8047</v>
       </c>
-      <c r="BA16" s="5" t="n">
+      <c r="BB16" s="5" t="n">
         <v>549</v>
       </c>
-      <c r="BB16" s="4" t="n">
+      <c r="BC16" s="4" t="n">
         <v>-0.438597160011436</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D17" s="4" t="n">
         <v>0.235</v>
@@ -3416,122 +3468,125 @@
       <c r="R17" s="5" t="n">
         <v>8334</v>
       </c>
-      <c r="S17" s="4" t="n">
+      <c r="S17" s="5" t="n">
+        <v>36039</v>
+      </c>
+      <c r="T17" s="4" t="n">
         <v>0.023</v>
       </c>
-      <c r="T17" s="4" t="n">
+      <c r="U17" s="4" t="n">
         <v>0.222</v>
       </c>
-      <c r="U17" s="5" t="n">
+      <c r="V17" s="5" t="n">
         <v>13274000</v>
       </c>
-      <c r="V17" s="5" t="n">
+      <c r="W17" s="5" t="n">
         <v>920996</v>
       </c>
-      <c r="W17" s="5"/>
-      <c r="X17" s="5" t="n">
+      <c r="X17" s="5"/>
+      <c r="Y17" s="5" t="n">
         <v>45250</v>
       </c>
-      <c r="Y17" s="5" t="n">
+      <c r="Z17" s="5" t="n">
         <v>20574</v>
       </c>
-      <c r="Z17" s="5" t="n">
+      <c r="AA17" s="5" t="n">
         <v>99.4</v>
       </c>
-      <c r="AA17" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="AB17" s="5" t="n">
+      <c r="AB17" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="AC17" s="5" t="n">
         <v>158300</v>
       </c>
-      <c r="AC17" s="5" t="n">
+      <c r="AD17" s="5" t="n">
         <v>102500</v>
       </c>
-      <c r="AD17" s="5" t="n">
+      <c r="AE17" s="5" t="n">
         <v>64290</v>
       </c>
-      <c r="AE17" s="5" t="n">
+      <c r="AF17" s="5" t="n">
         <v>218470</v>
       </c>
-      <c r="AF17" s="5" t="n">
+      <c r="AG17" s="5" t="n">
         <v>143200</v>
       </c>
-      <c r="AG17" s="5" t="n">
+      <c r="AH17" s="5" t="n">
         <v>90310</v>
       </c>
-      <c r="AH17" s="5" t="n">
+      <c r="AI17" s="5" t="n">
         <v>43</v>
       </c>
-      <c r="AI17" s="4" t="n">
+      <c r="AJ17" s="4" t="n">
         <v>0.2</v>
       </c>
-      <c r="AJ17" s="5" t="n">
+      <c r="AK17" s="5" t="n">
         <v>402024</v>
       </c>
-      <c r="AK17" s="5" t="n">
+      <c r="AL17" s="5" t="n">
         <v>29.1</v>
       </c>
-      <c r="AL17" s="5" t="n">
+      <c r="AM17" s="5" t="n">
         <v>39.5</v>
       </c>
-      <c r="AM17" s="5" t="n">
+      <c r="AN17" s="5" t="n">
         <v>339</v>
       </c>
-      <c r="AN17" s="5" t="n">
+      <c r="AO17" s="5" t="n">
         <v>29</v>
       </c>
-      <c r="AO17" s="4" t="n">
+      <c r="AP17" s="4" t="n">
         <v>0.13</v>
       </c>
-      <c r="AP17" s="4" t="n">
+      <c r="AQ17" s="4" t="n">
         <v>0.417</v>
       </c>
-      <c r="AQ17" s="4" t="n">
+      <c r="AR17" s="4" t="n">
         <v>0.815</v>
       </c>
-      <c r="AR17" s="5" t="n">
+      <c r="AS17" s="5" t="n">
         <v>267</v>
       </c>
-      <c r="AS17" s="5" t="n">
+      <c r="AT17" s="5" t="n">
         <v>5884</v>
       </c>
-      <c r="AT17" s="5" t="n">
+      <c r="AU17" s="5" t="n">
         <v>50482.43</v>
       </c>
-      <c r="AU17" s="4" t="n">
+      <c r="AV17" s="4" t="n">
         <v>0.463</v>
       </c>
-      <c r="AV17" s="4" t="n">
+      <c r="AW17" s="4" t="n">
         <v>0.538</v>
       </c>
-      <c r="AW17" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="AX17" s="4" t="n">
+      <c r="AX17" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="AY17" s="4" t="n">
         <v>0.7495</v>
       </c>
-      <c r="AY17" s="4" t="n">
+      <c r="AZ17" s="4" t="n">
         <v>0.6349</v>
       </c>
-      <c r="AZ17" s="4" t="n">
+      <c r="BA17" s="4" t="n">
         <v>0.7812</v>
       </c>
-      <c r="BA17" s="5" t="n">
+      <c r="BB17" s="5" t="n">
         <v>2397</v>
       </c>
-      <c r="BB17" s="4" t="n">
+      <c r="BC17" s="4" t="n">
         <v>-0.320368938767894</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D18" s="4" t="n">
         <v>0.276</v>
@@ -3578,122 +3633,125 @@
       <c r="R18" s="5" t="n">
         <v>8946</v>
       </c>
-      <c r="S18" s="4" t="n">
+      <c r="S18" s="5" t="n">
+        <v>40023</v>
+      </c>
+      <c r="T18" s="4" t="n">
         <v>0.041</v>
       </c>
-      <c r="T18" s="4" t="n">
+      <c r="U18" s="4" t="n">
         <v>0.259</v>
       </c>
-      <c r="U18" s="5" t="n">
+      <c r="V18" s="5" t="n">
         <v>23028800</v>
       </c>
-      <c r="V18" s="5" t="n">
+      <c r="W18" s="5" t="n">
         <v>693116</v>
       </c>
-      <c r="W18" s="5"/>
-      <c r="X18" s="5" t="n">
+      <c r="X18" s="5"/>
+      <c r="Y18" s="5" t="n">
         <v>57840</v>
       </c>
-      <c r="Y18" s="5" t="n">
+      <c r="Z18" s="5" t="n">
         <v>19422</v>
       </c>
-      <c r="Z18" s="5" t="n">
+      <c r="AA18" s="5" t="n">
         <v>228.7</v>
       </c>
-      <c r="AA18" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="AB18" s="5" t="n">
+      <c r="AB18" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="AC18" s="5" t="n">
         <v>51720</v>
       </c>
-      <c r="AC18" s="5" t="n">
+      <c r="AD18" s="5" t="n">
         <v>39010</v>
       </c>
-      <c r="AD18" s="5" t="n">
+      <c r="AE18" s="5" t="n">
         <v>22680</v>
       </c>
-      <c r="AE18" s="5" t="n">
+      <c r="AF18" s="5" t="n">
         <v>90860</v>
       </c>
-      <c r="AF18" s="5" t="n">
+      <c r="AG18" s="5" t="n">
         <v>66100</v>
       </c>
-      <c r="AG18" s="5" t="n">
+      <c r="AH18" s="5" t="n">
         <v>40000</v>
       </c>
-      <c r="AH18" s="5" t="n">
+      <c r="AI18" s="5" t="n">
         <v>41</v>
       </c>
-      <c r="AI18" s="4" t="n">
+      <c r="AJ18" s="4" t="n">
         <v>0.166</v>
       </c>
-      <c r="AJ18" s="5" t="n">
+      <c r="AK18" s="5" t="n">
         <v>317108</v>
       </c>
-      <c r="AK18" s="5" t="n">
+      <c r="AL18" s="5" t="n">
         <v>29.1</v>
       </c>
-      <c r="AL18" s="5" t="n">
+      <c r="AM18" s="5" t="n">
         <v>37.2</v>
       </c>
-      <c r="AM18" s="5" t="n">
+      <c r="AN18" s="5" t="n">
         <v>331</v>
       </c>
-      <c r="AN18" s="5" t="n">
+      <c r="AO18" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="AO18" s="4" t="n">
+      <c r="AP18" s="4" t="n">
         <v>0.263</v>
       </c>
-      <c r="AP18" s="4" t="n">
+      <c r="AQ18" s="4" t="n">
         <v>0.24</v>
       </c>
-      <c r="AQ18" s="4" t="n">
+      <c r="AR18" s="4" t="n">
         <v>0.624</v>
       </c>
-      <c r="AR18" s="5" t="n">
+      <c r="AS18" s="5" t="n">
         <v>241</v>
       </c>
-      <c r="AS18" s="5" t="n">
+      <c r="AT18" s="5" t="n">
         <v>7018</v>
       </c>
-      <c r="AT18" s="5" t="n">
+      <c r="AU18" s="5" t="n">
         <v>81510.55</v>
       </c>
-      <c r="AU18" s="4" t="n">
+      <c r="AV18" s="4" t="n">
         <v>0.371</v>
       </c>
-      <c r="AV18" s="4" t="n">
+      <c r="AW18" s="4" t="n">
         <v>0.538</v>
       </c>
-      <c r="AW18" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="AX18" s="4" t="n">
+      <c r="AX18" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="AY18" s="4" t="n">
         <v>0.8061</v>
       </c>
-      <c r="AY18" s="4" t="n">
+      <c r="AZ18" s="4" t="n">
         <v>0.6761</v>
       </c>
-      <c r="AZ18" s="4" t="n">
+      <c r="BA18" s="4" t="n">
         <v>0.8133</v>
       </c>
-      <c r="BA18" s="5" t="n">
+      <c r="BB18" s="5" t="n">
         <v>2748</v>
       </c>
-      <c r="BB18" s="4" t="n">
+      <c r="BC18" s="4" t="n">
         <v>-0.464097808395473</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D19" s="4" t="n">
         <v>0.196</v>
@@ -3740,122 +3798,125 @@
       <c r="R19" s="5" t="n">
         <v>7509</v>
       </c>
-      <c r="S19" s="4" t="n">
+      <c r="S19" s="5" t="n">
+        <v>28473</v>
+      </c>
+      <c r="T19" s="4" t="n">
         <v>0.047</v>
       </c>
-      <c r="T19" s="4" t="n">
+      <c r="U19" s="4" t="n">
         <v>0.257</v>
       </c>
-      <c r="U19" s="5" t="n">
+      <c r="V19" s="5" t="n">
         <v>57777600</v>
       </c>
-      <c r="V19" s="5" t="n">
+      <c r="W19" s="5" t="n">
         <v>1303981</v>
       </c>
-      <c r="W19" s="5"/>
-      <c r="X19" s="5" t="n">
+      <c r="X19" s="5"/>
+      <c r="Y19" s="5" t="n">
         <v>70760</v>
       </c>
-      <c r="Y19" s="5" t="n">
+      <c r="Z19" s="5" t="n">
         <v>58193</v>
       </c>
-      <c r="Z19" s="5" t="n">
+      <c r="AA19" s="5" t="n">
         <v>183.8</v>
       </c>
-      <c r="AA19" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="AB19" s="5" t="n">
+      <c r="AB19" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="AC19" s="5" t="n">
         <v>74050</v>
       </c>
-      <c r="AC19" s="5" t="n">
+      <c r="AD19" s="5" t="n">
         <v>69500</v>
       </c>
-      <c r="AD19" s="5" t="n">
+      <c r="AE19" s="5" t="n">
         <v>33270</v>
       </c>
-      <c r="AE19" s="5" t="n">
+      <c r="AF19" s="5" t="n">
         <v>130120</v>
       </c>
-      <c r="AF19" s="5" t="n">
+      <c r="AG19" s="5" t="n">
         <v>116000</v>
       </c>
-      <c r="AG19" s="5" t="n">
+      <c r="AH19" s="5" t="n">
         <v>58110</v>
       </c>
-      <c r="AH19" s="5" t="n">
+      <c r="AI19" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="AI19" s="4" t="n">
+      <c r="AJ19" s="4" t="n">
         <v>0.089</v>
       </c>
-      <c r="AJ19" s="5" t="n">
+      <c r="AK19" s="5" t="n">
         <v>168565</v>
       </c>
-      <c r="AK19" s="5" t="n">
+      <c r="AL19" s="5" t="n">
         <v>29.1</v>
       </c>
-      <c r="AL19" s="5" t="n">
+      <c r="AM19" s="5" t="n">
         <v>39.4</v>
       </c>
-      <c r="AM19" s="5" t="n">
+      <c r="AN19" s="5" t="n">
         <v>210</v>
       </c>
-      <c r="AN19" s="5" t="n">
+      <c r="AO19" s="5" t="n">
         <v>17</v>
       </c>
-      <c r="AO19" s="4" t="n">
+      <c r="AP19" s="4" t="n">
         <v>0.15</v>
       </c>
-      <c r="AP19" s="4" t="n">
+      <c r="AQ19" s="4" t="n">
         <v>0.366</v>
       </c>
-      <c r="AQ19" s="4" t="n">
+      <c r="AR19" s="4" t="n">
         <v>0.812</v>
       </c>
-      <c r="AR19" s="5" t="n">
+      <c r="AS19" s="5" t="n">
         <v>276</v>
       </c>
-      <c r="AS19" s="5" t="n">
+      <c r="AT19" s="5" t="n">
         <v>6952</v>
       </c>
-      <c r="AT19" s="5" t="n">
+      <c r="AU19" s="5" t="n">
         <v>64024.59</v>
       </c>
-      <c r="AU19" s="4" t="n">
+      <c r="AV19" s="4" t="n">
         <v>0.409</v>
       </c>
-      <c r="AV19" s="4" t="n">
+      <c r="AW19" s="4" t="n">
         <v>0.538</v>
       </c>
-      <c r="AW19" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="AX19" s="4" t="n">
+      <c r="AX19" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="AY19" s="4" t="n">
         <v>0.7611</v>
       </c>
-      <c r="AY19" s="4" t="n">
+      <c r="AZ19" s="4" t="n">
         <v>0.6445</v>
       </c>
-      <c r="AZ19" s="4" t="n">
+      <c r="BA19" s="4" t="n">
         <v>0.7944</v>
       </c>
-      <c r="BA19" s="5" t="n">
+      <c r="BB19" s="5" t="n">
         <v>1687</v>
       </c>
-      <c r="BB19" s="4" t="n">
+      <c r="BC19" s="4" t="n">
         <v>-0.23466140061554</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D20" s="4" t="n">
         <v>0.338</v>
@@ -3902,122 +3963,125 @@
       <c r="R20" s="5" t="n">
         <v>7629</v>
       </c>
-      <c r="S20" s="4" t="n">
+      <c r="S20" s="5" t="n">
+        <v>32229</v>
+      </c>
+      <c r="T20" s="4" t="n">
         <v>0.033</v>
       </c>
-      <c r="T20" s="4" t="n">
+      <c r="U20" s="4" t="n">
         <v>0.243</v>
       </c>
-      <c r="U20" s="5" t="n">
+      <c r="V20" s="5" t="n">
         <v>8446100</v>
       </c>
-      <c r="V20" s="5" t="n">
+      <c r="W20" s="5" t="n">
         <v>398629</v>
       </c>
-      <c r="W20" s="5"/>
-      <c r="X20" s="5" t="n">
+      <c r="X20" s="5"/>
+      <c r="Y20" s="5" t="n">
         <v>45470</v>
       </c>
-      <c r="Y20" s="5" t="n">
+      <c r="Z20" s="5" t="n">
         <v>17733</v>
       </c>
-      <c r="Z20" s="5" t="n">
+      <c r="AA20" s="5" t="n">
         <v>116</v>
       </c>
-      <c r="AA20" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="AB20" s="5" t="n">
+      <c r="AB20" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="AC20" s="5" t="n">
         <v>70030</v>
       </c>
-      <c r="AC20" s="5" t="n">
+      <c r="AD20" s="5" t="n">
         <v>61870</v>
       </c>
-      <c r="AD20" s="5" t="n">
+      <c r="AE20" s="5" t="n">
         <v>32380</v>
       </c>
-      <c r="AE20" s="5" t="n">
+      <c r="AF20" s="5" t="n">
         <v>112490</v>
       </c>
-      <c r="AF20" s="5" t="n">
+      <c r="AG20" s="5" t="n">
         <v>95380</v>
       </c>
-      <c r="AG20" s="5" t="n">
+      <c r="AH20" s="5" t="n">
         <v>51750</v>
       </c>
-      <c r="AH20" s="5" t="n">
+      <c r="AI20" s="5" t="n">
         <v>39</v>
       </c>
-      <c r="AI20" s="4" t="n">
+      <c r="AJ20" s="4" t="n">
         <v>0.193</v>
       </c>
-      <c r="AJ20" s="5" t="n">
+      <c r="AK20" s="5" t="n">
         <v>334551</v>
       </c>
-      <c r="AK20" s="5" t="n">
+      <c r="AL20" s="5" t="n">
         <v>29.2</v>
       </c>
-      <c r="AL20" s="5" t="n">
+      <c r="AM20" s="5" t="n">
         <v>39.7</v>
       </c>
-      <c r="AM20" s="5" t="n">
+      <c r="AN20" s="5" t="n">
         <v>532</v>
       </c>
-      <c r="AN20" s="5" t="n">
+      <c r="AO20" s="5" t="n">
         <v>43</v>
       </c>
-      <c r="AO20" s="4" t="n">
+      <c r="AP20" s="4" t="n">
         <v>0.283</v>
       </c>
-      <c r="AP20" s="4" t="n">
+      <c r="AQ20" s="4" t="n">
         <v>0.393</v>
       </c>
-      <c r="AQ20" s="4" t="n">
+      <c r="AR20" s="4" t="n">
         <v>0.697</v>
       </c>
-      <c r="AR20" s="5" t="n">
+      <c r="AS20" s="5" t="n">
         <v>310</v>
       </c>
-      <c r="AS20" s="5" t="n">
+      <c r="AT20" s="5" t="n">
         <v>12207</v>
       </c>
-      <c r="AT20" s="5" t="n">
+      <c r="AU20" s="5" t="n">
         <v>136974.62</v>
       </c>
-      <c r="AU20" s="4" t="n">
+      <c r="AV20" s="4" t="n">
         <v>0.459</v>
       </c>
-      <c r="AV20" s="4" t="n">
+      <c r="AW20" s="4" t="n">
         <v>0.538</v>
       </c>
-      <c r="AW20" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="AX20" s="4" t="n">
+      <c r="AX20" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="AY20" s="4" t="n">
         <v>0.8179</v>
       </c>
-      <c r="AY20" s="4" t="n">
+      <c r="AZ20" s="4" t="n">
         <v>0.6882</v>
       </c>
-      <c r="AZ20" s="4" t="n">
+      <c r="BA20" s="4" t="n">
         <v>0.8258</v>
       </c>
-      <c r="BA20" s="5" t="n">
+      <c r="BB20" s="5" t="n">
         <v>2165</v>
       </c>
-      <c r="BB20" s="4" t="n">
+      <c r="BC20" s="4" t="n">
         <v>-0.405758612895935</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D21" s="6" t="n">
         <v>0.316</v>
@@ -4064,117 +4128,120 @@
       <c r="R21" s="7" t="n">
         <v>39310</v>
       </c>
-      <c r="S21" s="6" t="n">
+      <c r="S21" s="7" t="n">
+        <v>154436</v>
+      </c>
+      <c r="T21" s="6" t="n">
         <v>0.043</v>
       </c>
-      <c r="T21" s="6" t="n">
+      <c r="U21" s="6" t="n">
         <v>0.284</v>
       </c>
-      <c r="U21" s="7" t="n">
+      <c r="V21" s="7" t="n">
         <v>102900</v>
       </c>
-      <c r="V21" s="7" t="n">
+      <c r="W21" s="7" t="n">
         <v>357940</v>
       </c>
-      <c r="W21" s="7" t="n">
+      <c r="X21" s="7" t="n">
         <v>0.66</v>
       </c>
-      <c r="X21" s="7" t="n">
+      <c r="Y21" s="7" t="n">
         <v>60470</v>
       </c>
-      <c r="Y21" s="7" t="n">
+      <c r="Z21" s="7" t="n">
         <v>50483</v>
       </c>
-      <c r="Z21" s="7" t="n">
+      <c r="AA21" s="7" t="n">
         <v>22.1</v>
       </c>
-      <c r="AA21" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="AB21" s="7" t="n">
+      <c r="AB21" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC21" s="7" t="n">
         <v>626480</v>
       </c>
-      <c r="AC21" s="7" t="n">
+      <c r="AD21" s="7" t="n">
         <v>433800</v>
       </c>
-      <c r="AD21" s="7" t="n">
+      <c r="AE21" s="7" t="n">
         <v>257810</v>
       </c>
-      <c r="AE21" s="7" t="n">
+      <c r="AF21" s="7" t="n">
         <v>1079790</v>
       </c>
-      <c r="AF21" s="7" t="n">
+      <c r="AG21" s="7" t="n">
         <v>727630</v>
       </c>
-      <c r="AG21" s="7" t="n">
+      <c r="AH21" s="7" t="n">
         <v>439950</v>
       </c>
-      <c r="AH21" s="7" t="n">
+      <c r="AI21" s="7" t="n">
         <v>677</v>
       </c>
-      <c r="AI21" s="6" t="n">
+      <c r="AJ21" s="6" t="n">
         <v>0.676</v>
       </c>
-      <c r="AJ21" s="7" t="n">
+      <c r="AK21" s="7" t="n">
         <v>6061280</v>
       </c>
-      <c r="AK21" s="7" t="n">
+      <c r="AL21" s="7" t="n">
         <v>31.1</v>
       </c>
-      <c r="AL21" s="7" t="n">
+      <c r="AM21" s="7" t="n">
         <v>40.4</v>
       </c>
-      <c r="AM21" s="7" t="n">
+      <c r="AN21" s="7" t="n">
         <v>1294</v>
       </c>
-      <c r="AN21" s="7" t="n">
+      <c r="AO21" s="7" t="n">
         <v>177</v>
       </c>
-      <c r="AO21" s="6" t="n">
+      <c r="AP21" s="6" t="n">
         <v>0.183</v>
       </c>
-      <c r="AP21" s="6" t="n">
+      <c r="AQ21" s="6" t="n">
         <v>0.463</v>
       </c>
-      <c r="AQ21" s="6" t="n">
+      <c r="AR21" s="6" t="n">
         <v>0.825</v>
       </c>
-      <c r="AR21" s="7" t="n">
+      <c r="AS21" s="7" t="n">
         <v>181</v>
       </c>
-      <c r="AS21" s="7" t="n">
+      <c r="AT21" s="7" t="n">
         <v>2487</v>
       </c>
-      <c r="AT21" s="7" t="n">
+      <c r="AU21" s="7" t="n">
         <v>9483.55</v>
       </c>
-      <c r="AU21" s="6" t="n">
+      <c r="AV21" s="6" t="n">
         <v>0.327</v>
       </c>
-      <c r="AV21" s="6" t="n">
+      <c r="AW21" s="6" t="n">
         <v>0.538</v>
       </c>
-      <c r="AW21" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="AX21" s="6" t="n">
+      <c r="AX21" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="AY21" s="6" t="n">
         <v>0.8266</v>
       </c>
-      <c r="AY21" s="6" t="n">
+      <c r="AZ21" s="6" t="n">
         <v>0.7048</v>
       </c>
-      <c r="AZ21" s="6" t="n">
+      <c r="BA21" s="6" t="n">
         <v>0.8074</v>
       </c>
-      <c r="BA21" s="7" t="n">
+      <c r="BB21" s="7" t="n">
         <v>4098</v>
       </c>
-      <c r="BB21" s="6" t="n">
+      <c r="BC21" s="6" t="n">
         <v>0.0272380558626413</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BB1"/>
+  <autoFilter ref="A1:BC1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>

</xml_diff>